<commit_message>
sync: Vollstaendige Konsolidierung aller Projekt-Dateien gemaess den 11 Kriterien der Schulcheckliste
</commit_message>
<xml_diff>
--- a/Anforderungsprotokoll_Arduino_Teststand_v1.1.xlsx
+++ b/Anforderungsprotokoll_Arduino_Teststand_v1.1.xlsx
@@ -124,7 +124,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -165,11 +165,79 @@
         <color rgb="00D0D7DE"/>
       </top>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D0D7DE"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D0D7DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D7DE"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D0D7DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D7DE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D7DE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D0D7DE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D7DE"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D0D7DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D7DE"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001B365D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D0D7DE"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001B365D"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -229,6 +297,11 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -620,6 +693,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2x Arduino Uno R4 (Renesas RA4M1) | Systemebene (Blackbox-Betrachtung)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -628,11 +708,11 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>2× Arduino Uno R3 (ATmega328P) | Systemebene (Blackbox-Betrachtung)</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
+          <t>01.09.2026 / Version 1.2 (Abgestimmt auf die 11 Kriterien der Schulcheckliste)</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="n"/>
+      <c r="D4" s="28" t="n"/>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Ersteller / Team:</t>
@@ -643,7 +723,7 @@
           <t>Projektteam Fachschule Technik</t>
         </is>
       </c>
-      <c r="G4" s="5" t="n"/>
+      <c r="G4" s="28" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -656,8 +736,8 @@
           <t>25.08.2026 / Version 1.1 (Erweitert um Systemkriterien)</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
+      <c r="C5" s="27" t="n"/>
+      <c r="D5" s="28" t="n"/>
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Status / Freigabe:</t>
@@ -668,7 +748,7 @@
           <t>In Abstimmung / Diskussionsgrundlage</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n"/>
+      <c r="G5" s="28" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -681,8 +761,8 @@
           <t>Δt im Versuch zu evaluieren (Richtwert: 50 ms)</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
+      <c r="C6" s="27" t="n"/>
+      <c r="D6" s="28" t="n"/>
       <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Filterung:</t>
@@ -693,8 +773,9 @@
           <t>Gleitender Mittelwert (N = 10 Samples)</t>
         </is>
       </c>
-      <c r="G6" s="5" t="n"/>
-    </row>
+      <c r="G6" s="28" t="n"/>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
@@ -745,17 +826,17 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Analoge Eingangserfassung</t>
+          <t>Analoge Eingangserfassung: Kontinuierliche Erfassung eines analogen DC-Signals (0..5,00 V) ueber 10-Bit-Quantisierung (0..1023 Digits) an Analogeingang A0.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Linearitaetsfehler &lt;= +-2 LSB</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>Erfassung analoger Signale über 10-Bit-ADC (0..1023 Digits, 0..5 V Messbereich) an Kanal A0</t>
+          <t>Kalibrierte DC-Spannungsquelle &amp; Digitalmultimeter (DMM)</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -782,17 +863,17 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Entprellung / Rauschunterdrückung</t>
+          <t>Rauschunterdrueckung &amp; Glaettung: Zeitdiskrete Glaettung des Eingangssignals mittels gleitendem arithmetischem Mittelwert ueber genau N=10 aufeinanderfolgende Messpunkte.</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Abtastintervall dt=50ms +- 2ms (20 Hz Abtastrate)</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Gleitender arithmetischer Mittelwert über N = 10 Samples. Zeitintervall Δt parametrierbar.</t>
+          <t>Signalvergleich Roh- vs. Filterwert im Arduino Serial Plotter</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
@@ -819,17 +900,17 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Erweiterbarkeit der Eingangskanäle</t>
+          <t>Erweiterbarkeit der Eingangskanaele: Systemarchitektur muss fuer die synchrone Erfassung von bis zu 6 analogen Signalgebern modular erweiterbar sein.</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>Hardware- und Softwaredesign unterstuetzt Kanaele A0-A5</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>System- und Schnittstellenarchitektur ausgelegt für bis zu 6 analoge Kanäle (A0–A5)</t>
+          <t>Funktionstest mit bis zu 6 analogen Signalgebern</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -856,17 +937,17 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Zyklische Bus-Datenübertragung</t>
+          <t>Zyklische Bus-Datenuebertragung: Unaufgeforderte, zyklische Uebertragung des berechneten Messwerts und des Rohwerts ueber eine serielle Punkt-zu-Punkt-Busverbindung.</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Uebertragungsrate f_bus &gt;= 10 Hz (Intervall &lt;= 100ms), 9600 Baud 8N1, Telegramm &lt;VAL:xxxx;RAW:xxxx&gt;</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Zyklische Übertragung des Mittelwerts via UART-Bus. Aktualisierungsrate f_bus &gt;= 10 Hz.</t>
+          <t>Logikanalysator / Serial-Monitor-Trace mit Zeitstempeln</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
@@ -893,17 +974,17 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Bus-Timeout &amp; Verbindungsüberwachung</t>
+          <t>Bus-Timeout &amp; Verbindungsueberwachung: Selbststaendige Erkennung eines Kommunikationsausfalls mit optischer Warnanzeige und automatischem Wiederanlauf bei Signalrueckkehr.</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Wechsel in Fehlermodus bei Ausfall &gt; 2.0 s; Wiederanlaufzeit &lt;= 200 ms</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>Erkennung von Übertragungsunterbrechungen. Fehlermeldung auf LCD bei Telegrammausfall &gt; 2 s.</t>
+          <t>Unterbrechung der RX/TX-Signalleitung im laufenden Betrieb</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -930,17 +1011,17 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>LC-Display Ansteuerung</t>
+          <t>Messwert-Visualisierung: Strukturierte 4-zeilige Monospace-Textanzeige zur simultanen Darstellung von Binaerwert, Dezimalwert, Abweichung und Systemstatus.</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>4 Zeilen a 20 Zeichen, synchrone 2-Draht-Ansteuerung (100 kHz)</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Anbindung eines HD44780-kompatiblen LCDs via I2C-Schnittstelle (PCF8574 Backpack)</t>
+          <t>I2C-Bus-Scan / Hardwaretest mit Oszilloskop</t>
         </is>
       </c>
       <c r="F14" s="11" t="inlineStr">
@@ -967,17 +1048,17 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Binäre Messwertdarstellung</t>
+          <t>Binaere Messwertdarstellung: Formatierte 10-Bit-Binaerausgabe mit fuehrenden Nullen und optischer 4-Bit-Nibble-Trennung auf Zeile 1 des Displays.</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Formatierung exakt BIN: bb bbbb bbbb (0..1023)</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>10-Bit-Messwert im Binärformat (führende Nullen, Nibble-Trennung bei Displays &gt;= 20 Zeichen)</t>
+          <t>Sichtpruefung der LCD-Anzeige ueber gesamten Stellbereich</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -1004,17 +1085,17 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Messwert-Aktualisierung (Hold-Trigger)</t>
+          <t>Messwert-Uebernahme (Hold-Funktion): Aktualisierung der Displayanzeige ausschliesslich bei gezielter Betaetigung des Bedientasters; dauerhaftes Halten des Anzeigewerts bis zum Folgeimpuls.</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Sichere Unterdrueckung von Kontaktprellen mit Entprellzeit t_deb &gt;= 50 ms</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Anzeige-Aktualisierung nur bei Tastenbetätigung. Entprellzeit t_deb &gt;= 50 ms.</t>
+          <t>Prellpruefung / Funktionstest mit Oszilloskop am Tastereingang</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
@@ -1041,17 +1122,17 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Reaktionszeit HMI-Aktualisierung</t>
+          <t>Reaktionszeit HMI-Aktualisierung: Zeitverzoegerung zwischen Tasterbetaetigung (fallende Flanke) und vollstaendiger Aktualisierung des Displayinhalts.</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Gesamtlatenzzeit t_lat &lt;= 100 ms</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>Latenz zwischen Tasterbetätigung und Display-Aktualisierung t_lat &lt;= 100 ms</t>
+          <t>2-Kanal-Oszilloskop (Trigger Flanke Taster -&gt; I2C Paket)</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
@@ -1078,17 +1159,17 @@
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Definiertes Initialisierungsverhalten</t>
+          <t>Definiertes Initialisierungsverhalten: Deterministischer Kaltstart-Ablauf mit Begruessungsanzeige, Filter-Vorbefuellung und Einnahme eines sicheren Wartezustands.</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Boot-Screen 2.0 s +- 0.1 s, Vorbefuellung N=10, Status: MOD: WAIT TASTE</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Nach Power-On: Boot-Meldung, Puffer-Füllroutine, definierter Wartezustand bis zum ersten Tastendruck</t>
+          <t>Einschaltpruefung / Kaltstart-Zyklus mit Netztrennung</t>
         </is>
       </c>
       <c r="F18" s="11" t="inlineStr">
@@ -1115,17 +1196,17 @@
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Grenzwertüberwachung (Sprung &gt; 70 %)</t>
+          <t>Plausibilitaets- &amp; Grenzwertueberwachung: Erkennung und optische Signalisierung unplausibler Signalspruenge (&gt;= 70%) im Vergleich zum vorhergehenden Messwert.</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Optischer Alarm DEV: +xx.x% [ALARM] bei |Delta_rel| &gt;= 70.0%; Nullpunkt |Delta| &gt;= 50 Digits</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>Optischer LCD-Alarm bei |Wert(k) - Wert(k-1)| &gt;= 0.70 * Wert(k-1). Abfangung von Wert(k-1) = 0.</t>
+          <t>Sprungantwort-Test mit Spannungssprung am Poti</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
@@ -1152,17 +1233,17 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Alarm-Rücksetzung / Statusquittierung</t>
+          <t>Alarm-Ruecksetzung &amp; Quittierung: Der optische Alarmzustand bleibt solange aktiv, bis ein neuer Messwert innerhalb des zulaessigen Toleranzbereichs (&lt; 70%) per Taster bestaetigt wird.</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Ruecksetzung des Alarmstatus auf [OK] bei nachfolgendem Messwert im Nennbereich</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>Alarm bleibt aktiv, bis ein neuer Messwert innerhalb des Toleranzbereichs liegt oder quittiert wird</t>
+          <t>Stufentest mit Rueckkehr in den Toleranzbereich</t>
         </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
@@ -1189,17 +1270,17 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Direkter Zugriff zur Weiterverarbeitung</t>
+          <t>Messwert- &amp; Referenzwertpufferung: Unterbrechungsfreie Vorhaltung von aktuellem Messwert, vorhergehendem Referenzwert und Filterhistorie zur Laufzeit.</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Verzoegerungsfreie Bereitstellung aller Operanden im Arbeitsspeicher</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>Vorhaltung von aktuellem Wert, Vorgängerwert und Systemstatus im flüchtigen SRAM</t>
+          <t>Code-Review &amp; Verifikation des deterministischen Speicherverhaltens</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -1226,17 +1307,17 @@
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Betriebsspannung &amp; Bezugspotenzial</t>
+          <t>Betriebsspannung &amp; Signalintegritaet: Sichere Funktion bei Nennspannung +5.0V DC mit Schutz gegen offene/schwebende Eingangspotenziale.</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Spannungsbereich +5.0V DC +- 5%, definierte High-Pegel an Schalteingaengen</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>+5 V DC Versorgung über USB/Netzteil. Zwingendes gemeinsames Bezugspotenzial (GND-Kopplung)</t>
+          <t>DMM-Spannungsmessung &amp; Verifikationspruefung offener Pins</t>
         </is>
       </c>
       <c r="F22" s="11" t="inlineStr">
@@ -1263,17 +1344,17 @@
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Betriebsumgebung &amp; Schutz</t>
+          <t>Betriebsumgebung &amp; Laborbetrieb: Zuverlaessiger Betrieb unter Standard-Labor- und Schulungsbedingungen.</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>Betriebsbereich 10..40 C, rel. Feuchte 20%..80%, IP20</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>Betriebsbereich: 10 °C bis 40 °C, Laborumgebung, Schutz vor Kurzschluss und unbeschalteten Eingängen</t>
+          <t>Sicht- und Funktionspruefung unter Laborbedingungen</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1287,6 +1368,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
@@ -1294,6 +1376,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
@@ -1306,9 +1389,14 @@
         </is>
       </c>
     </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="15" t="n"/>
+      <c r="B29" s="29" t="n"/>
+      <c r="C29" s="29" t="n"/>
       <c r="E29" s="15" t="n"/>
+      <c r="F29" s="29" t="n"/>
+      <c r="G29" s="29" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -2060,14 +2148,14 @@
           <t>Beispielanzeige (Monospace)</t>
         </is>
       </c>
-      <c r="C16" s="24" t="n"/>
+      <c r="C16" s="30" t="n"/>
       <c r="D16" s="23" t="inlineStr">
         <is>
           <t>Bedeutung / Feldfunktion</t>
         </is>
       </c>
-      <c r="E16" s="24" t="n"/>
-      <c r="F16" s="24" t="n"/>
+      <c r="E16" s="31" t="n"/>
+      <c r="F16" s="30" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -2080,14 +2168,14 @@
           <t>BIN: 00 1111 1111</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n"/>
+      <c r="C17" s="28" t="n"/>
       <c r="D17" s="21" t="inlineStr">
         <is>
           <t>10-Bit Binärwert mit 4er-Nibble-Gruppierung</t>
         </is>
       </c>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
+      <c r="E17" s="27" t="n"/>
+      <c r="F17" s="28" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -2100,14 +2188,14 @@
           <t>DEC: 1023 (Avg:10)</t>
         </is>
       </c>
-      <c r="C18" s="5" t="n"/>
+      <c r="C18" s="28" t="n"/>
       <c r="D18" s="22" t="inlineStr">
         <is>
           <t>Dezimalwert und Filterangabe</t>
         </is>
       </c>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
+      <c r="E18" s="27" t="n"/>
+      <c r="F18" s="28" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
@@ -2120,14 +2208,14 @@
           <t xml:space="preserve">DEV: +00.0% [OK]  </t>
         </is>
       </c>
-      <c r="C19" s="5" t="n"/>
+      <c r="C19" s="28" t="n"/>
       <c r="D19" s="21" t="inlineStr">
         <is>
           <t>Abweichungsüberwachung (|Δ| &lt; 70%)</t>
         </is>
       </c>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
+      <c r="E19" s="27" t="n"/>
+      <c r="F19" s="28" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
@@ -2140,14 +2228,14 @@
           <t xml:space="preserve">MOD: HOLD [TASTE] </t>
         </is>
       </c>
-      <c r="C20" s="5" t="n"/>
+      <c r="C20" s="28" t="n"/>
       <c r="D20" s="22" t="inlineStr">
         <is>
           <t>Statusanzeige: Aktualisierung nur auf Tastendruck</t>
         </is>
       </c>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n"/>
+      <c r="E20" s="27" t="n"/>
+      <c r="F20" s="28" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="13">

</xml_diff>